<commit_message>
find p values for backward euler and implicit midpoint methods
</commit_message>
<xml_diff>
--- a/Local Truncation Error Scaling vs. Step Size Table.xlsx
+++ b/Local Truncation Error Scaling vs. Step Size Table.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olincollege-my.sharepoint.com/personal/mepstein_olin_edu/Documents/Desktop/Applied Math/mth3199_assignment3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="11_F25DC773A252ABDACC10482CB99841445ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A085A5F3-99F7-4F86-9D36-00BB00989BBA}"/>
+  <xr:revisionPtr revIDLastSave="146" documentId="11_F25DC773A252ABDACC10482CB99841445ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{645A746A-F7C7-4E89-B52A-C9B80FD9BFA7}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Local Truncation Error Scaling" sheetId="1" r:id="rId1"/>
+    <sheet name="Global Truncation Error Scaling" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="13">
   <si>
     <t>Method</t>
   </si>
@@ -52,6 +53,18 @@
   </si>
   <si>
     <t>Local Truncation Error Scaling vs. Step Size Table</t>
+  </si>
+  <si>
+    <t>Global  Truncation Error Scaling vs. Step Size Table</t>
+  </si>
+  <si>
+    <t>diff</t>
+  </si>
+  <si>
+    <t>euler</t>
+  </si>
+  <si>
+    <t>midpoint</t>
   </si>
 </sst>
 </file>
@@ -125,22 +138,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -156,6 +168,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -431,73 +447,157 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
+      <c r="B3" s="4">
+        <v>1.0150999999999999</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5">
-        <v>6.1000000000000004E-3</v>
-      </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
+      <c r="B4" s="4">
+        <v>1.9968999999999999</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
+      <c r="B5" s="4">
+        <v>1.9208000000000001</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="5">
-        <v>6.3E-3</v>
-      </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
+      <c r="B6" s="4">
+        <v>2.9990999999999999</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
+      <c r="B7" s="4">
+        <v>2.9554</v>
+      </c>
+      <c r="C7" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44F93896-2EAF-4F6E-934F-AB5BFF4B3365}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="20.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4">
+        <v>-0.99939999999999996</v>
+      </c>
+      <c r="C4" s="4"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4">
+        <v>-2.0489000000000002</v>
+      </c>
+      <c r="C6" s="4"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
finish p value tables for error scaling vs step size
</commit_message>
<xml_diff>
--- a/Local Truncation Error Scaling vs. Step Size Table.xlsx
+++ b/Local Truncation Error Scaling vs. Step Size Table.xlsx
@@ -8,25 +8,38 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olincollege-my.sharepoint.com/personal/mepstein_olin_edu/Documents/Desktop/Applied Math/mth3199_assignment3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="146" documentId="11_F25DC773A252ABDACC10482CB99841445ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{645A746A-F7C7-4E89-B52A-C9B80FD9BFA7}"/>
+  <xr:revisionPtr revIDLastSave="204" documentId="11_F25DC773A252ABDACC10482CB99841445ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D246AB62-64DC-4E77-8254-5C55B5862599}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Local Truncation Error Scaling" sheetId="1" r:id="rId1"/>
     <sheet name="Global Truncation Error Scaling" sheetId="3" r:id="rId2"/>
+    <sheet name="Local Truncation Error Scaling " sheetId="4" r:id="rId3"/>
+    <sheet name="Global Truncation Scaling vs. R" sheetId="5" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="13">
   <si>
     <t>Method</t>
   </si>
@@ -58,13 +71,13 @@
     <t>Global  Truncation Error Scaling vs. Step Size Table</t>
   </si>
   <si>
-    <t>diff</t>
-  </si>
-  <si>
-    <t>euler</t>
-  </si>
-  <si>
-    <t>midpoint</t>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Global Truncation Error Scaling vs. Rate Function Calls Table</t>
+  </si>
+  <si>
+    <t>Local Truncation Error Scaling vs. Rate Function Calls Table</t>
   </si>
 </sst>
 </file>
@@ -473,8 +486,8 @@
       <c r="B3" s="4">
         <v>1.0150999999999999</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>10</v>
+      <c r="C3" s="4">
+        <v>1</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
@@ -486,8 +499,8 @@
       <c r="B4" s="4">
         <v>1.9968999999999999</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>11</v>
+      <c r="C4" s="4">
+        <v>2</v>
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
@@ -499,7 +512,9 @@
       <c r="B5" s="4">
         <v>1.9208000000000001</v>
       </c>
-      <c r="C5" s="4"/>
+      <c r="C5" s="4">
+        <v>2</v>
+      </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
     </row>
@@ -510,8 +525,8 @@
       <c r="B6" s="4">
         <v>2.9990999999999999</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>12</v>
+      <c r="C6" s="4">
+        <v>3</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -523,13 +538,16 @@
       <c r="B7" s="4">
         <v>2.9554</v>
       </c>
-      <c r="C7" s="4"/>
+      <c r="C7" s="4">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -564,40 +582,239 @@
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
+      <c r="B3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="4">
-        <v>-0.99939999999999996</v>
-      </c>
-      <c r="C4" s="4"/>
+        <v>0.99939999999999996</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1.0422</v>
+      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
+      <c r="B5" s="4">
+        <v>0.99960000000000004</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1.0422</v>
+      </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="4">
-        <v>-2.0489000000000002</v>
-      </c>
-      <c r="C6" s="4"/>
+        <v>2.0489000000000002</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1.9984</v>
+      </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
+      <c r="B7" s="4">
+        <v>1.9984999999999999</v>
+      </c>
+      <c r="C7" s="4">
+        <v>1.9984</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2524A753-95C8-4813-9511-CDEE9F45E7AC}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.109375" customWidth="1"/>
+    <col min="3" max="3" width="27" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4">
+        <v>0.99939999999999996</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1.0422</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4">
+        <v>0.99960000000000004</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1.0422</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4">
+        <v>2.0489000000000002</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1.9984</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4">
+        <v>1.9984999999999999</v>
+      </c>
+      <c r="C7" s="4">
+        <v>1.9984</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47261768-45E5-45A4-9E8E-EA64B3B092EA}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4">
+        <v>0.99939999999999996</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1.0422</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4">
+        <v>0.99960000000000004</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1.0422</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4">
+        <v>2.0489000000000002</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1.9984</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4">
+        <v>1.9984999999999999</v>
+      </c>
+      <c r="C7" s="4">
+        <v>1.9984</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
add rate function calls tables
</commit_message>
<xml_diff>
--- a/Local Truncation Error Scaling vs. Step Size Table.xlsx
+++ b/Local Truncation Error Scaling vs. Step Size Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olincollege-my.sharepoint.com/personal/mepstein_olin_edu/Documents/Desktop/Applied Math/mth3199_assignment3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="204" documentId="11_F25DC773A252ABDACC10482CB99841445ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D246AB62-64DC-4E77-8254-5C55B5862599}"/>
+  <xr:revisionPtr revIDLastSave="239" documentId="11_F25DC773A252ABDACC10482CB99841445ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{207B3265-A8CD-4F0F-AA3F-6AA294208D28}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6144" yWindow="0" windowWidth="16992" windowHeight="12336" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Local Truncation Error Scaling" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="13">
   <si>
     <t>Method</t>
   </si>
@@ -674,11 +674,11 @@
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>10</v>
+      <c r="B3" s="4">
+        <v>1.0166999999999999</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0.99990000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -686,10 +686,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="4">
-        <v>0.99939999999999996</v>
+        <v>1.9964999999999999</v>
       </c>
       <c r="C4" s="4">
-        <v>1.0422</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -697,10 +697,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="4">
-        <v>0.99960000000000004</v>
+        <v>1.9131</v>
       </c>
       <c r="C5" s="4">
-        <v>1.0422</v>
+        <v>1.9992000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -708,10 +708,10 @@
         <v>4</v>
       </c>
       <c r="B6" s="4">
-        <v>2.0489000000000002</v>
+        <v>2.9988999999999999</v>
       </c>
       <c r="C6" s="4">
-        <v>1.9984</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -719,10 +719,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="4">
-        <v>1.9984999999999999</v>
+        <v>2.9508000000000001</v>
       </c>
       <c r="C7" s="4">
-        <v>1.9984</v>
+        <v>2.9998</v>
       </c>
     </row>
   </sheetData>
@@ -730,6 +730,7 @@
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -739,8 +740,8 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="2" max="2" width="26.44140625" customWidth="1"/>
+    <col min="3" max="3" width="28.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.35">
@@ -777,10 +778,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="4">
-        <v>0.99939999999999996</v>
+        <v>0.99909999999999999</v>
       </c>
       <c r="C4" s="4">
-        <v>1.0422</v>
+        <v>1.0479000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -788,10 +789,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="4">
-        <v>0.99960000000000004</v>
+        <v>1.0002</v>
       </c>
       <c r="C5" s="4">
-        <v>1.0422</v>
+        <v>0.95399999999999996</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -799,10 +800,10 @@
         <v>4</v>
       </c>
       <c r="B6" s="4">
-        <v>2.0489000000000002</v>
+        <v>2.0548000000000002</v>
       </c>
       <c r="C6" s="4">
-        <v>1.9984</v>
+        <v>1.9997</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -810,10 +811,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="4">
-        <v>1.9984999999999999</v>
+        <v>1.9998</v>
       </c>
       <c r="C7" s="4">
-        <v>1.9984</v>
+        <v>1.9994000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -821,5 +822,6 @@
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update tables and fix stability plots
</commit_message>
<xml_diff>
--- a/Local Truncation Error Scaling vs. Step Size Table.xlsx
+++ b/Local Truncation Error Scaling vs. Step Size Table.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olincollege-my.sharepoint.com/personal/mepstein_olin_edu/Documents/Desktop/Applied Math/mth3199_assignment3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="239" documentId="11_F25DC773A252ABDACC10482CB99841445ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{207B3265-A8CD-4F0F-AA3F-6AA294208D28}"/>
+  <xr:revisionPtr revIDLastSave="244" documentId="11_F25DC773A252ABDACC10482CB99841445ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A5E67C7-D2F1-4260-AB74-D358B345749B}"/>
   <bookViews>
-    <workbookView xWindow="6144" yWindow="0" windowWidth="16992" windowHeight="12336" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Local Truncation Error Scaling" sheetId="1" r:id="rId1"/>
     <sheet name="Global Truncation Error Scaling" sheetId="3" r:id="rId2"/>
-    <sheet name="Local Truncation Error Scaling " sheetId="4" r:id="rId3"/>
-    <sheet name="Global Truncation Scaling vs. R" sheetId="5" r:id="rId4"/>
+    <sheet name="Global Truncation Scaling vs. R" sheetId="5" r:id="rId3"/>
+    <sheet name="Local Truncation Error Scaling " sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="12">
   <si>
     <t>Method</t>
   </si>
@@ -69,9 +69,6 @@
   </si>
   <si>
     <t>Global  Truncation Error Scaling vs. Step Size Table</t>
-  </si>
-  <si>
-    <t>N/A</t>
   </si>
   <si>
     <t>Global Truncation Error Scaling vs. Rate Function Calls Table</t>
@@ -553,7 +550,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44F93896-2EAF-4F6E-934F-AB5BFF4B3365}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.88671875" bestFit="1" customWidth="1"/>
@@ -580,21 +577,21 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>10</v>
+        <v>2</v>
+      </c>
+      <c r="B3" s="4">
+        <v>0.99939999999999996</v>
+      </c>
+      <c r="C3" s="4">
+        <v>1.0422</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" s="4">
-        <v>0.99939999999999996</v>
+        <v>0.99960000000000004</v>
       </c>
       <c r="C4" s="4">
         <v>1.0422</v>
@@ -602,34 +599,23 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" s="4">
-        <v>0.99960000000000004</v>
+        <v>2.0489000000000002</v>
       </c>
       <c r="C5" s="4">
-        <v>1.0422</v>
+        <v>1.9984</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" s="4">
-        <v>2.0489000000000002</v>
+        <v>1.9984999999999999</v>
       </c>
       <c r="C6" s="4">
-        <v>1.9984</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="4">
-        <v>1.9984999999999999</v>
-      </c>
-      <c r="C7" s="4">
         <v>1.9984</v>
       </c>
     </row>
@@ -643,6 +629,87 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47261768-45E5-45A4-9E8E-EA64B3B092EA}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.44140625" customWidth="1"/>
+    <col min="3" max="3" width="28.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4">
+        <v>0.99909999999999999</v>
+      </c>
+      <c r="C3" s="4">
+        <v>1.0479000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4">
+        <v>1.0002</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0.95399999999999996</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4">
+        <v>2.0548000000000002</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1.9997</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4">
+        <v>1.9998</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1.9994000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2524A753-95C8-4813-9511-CDEE9F45E7AC}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -654,7 +721,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -723,98 +790,6 @@
       </c>
       <c r="C7" s="4">
         <v>2.9998</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47261768-45E5-45A4-9E8E-EA64B3B092EA}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.44140625" customWidth="1"/>
-    <col min="3" max="3" width="28.5546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="4">
-        <v>0.99909999999999999</v>
-      </c>
-      <c r="C4" s="4">
-        <v>1.0479000000000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="4">
-        <v>1.0002</v>
-      </c>
-      <c r="C5" s="4">
-        <v>0.95399999999999996</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="4">
-        <v>2.0548000000000002</v>
-      </c>
-      <c r="C6" s="4">
-        <v>1.9997</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="4">
-        <v>1.9998</v>
-      </c>
-      <c r="C7" s="4">
-        <v>1.9994000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>